<commit_message>
docs: Add comprehensive SIH 2026 documentation and sync call response logs
</commit_message>
<xml_diff>
--- a/responses.xlsx
+++ b/responses.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,228 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:14:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:23:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Specialist Consultation</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Brain and Nerve Specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-24 12:30:06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pregnancy Care</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-29 20:16:29</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Specialist Consultation</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Heart Specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:52:40</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Specialist Consultation</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Heart Specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-29 21:54:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+17372508034</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>